<commit_message>
chore: snapshot do WAVOIP para análise
</commit_message>
<xml_diff>
--- a/planilha_teste.xlsx
+++ b/planilha_teste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caio.vicente\Desktop\wavoip att\WAVOIP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{04A48E9A-A060-4CD1-9600-DD734ADCDD76}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986647B2-9C8A-4384-BEB9-533453E9C4F2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,11 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>CPF</t>
   </si>
@@ -33,9 +32,6 @@
   </si>
   <si>
     <t>KARINE LEANDRA ANTUNES REGO</t>
-  </si>
-  <si>
-    <t>JP</t>
   </si>
 </sst>
 </file>
@@ -398,7 +394,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -424,18 +420,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>5521966491519</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>17623241729</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>5521981811077</v>
+        <v>5521984354821</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: suporte a txt, otimizacao do dashboard e edicao de tabulacoes
</commit_message>
<xml_diff>
--- a/planilha_teste.xlsx
+++ b/planilha_teste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caio.vicente\Desktop\wavoip att\WAVOIP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986647B2-9C8A-4384-BEB9-533453E9C4F2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52CADCEE-A13B-42DA-822B-661CECCBF991}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -420,7 +420,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>5521984354821</v>
+        <v>5521981811077</v>
       </c>
     </row>
   </sheetData>

</xml_diff>